<commit_message>
revised and added for the thematic relations
</commit_message>
<xml_diff>
--- a/Overall Files/Relation.xlsx
+++ b/Overall Files/Relation.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minsik/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3486D412-6BB4-3A4E-97E4-A0FCA1E84443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73879C06-5509-4C48-B9C9-F72017519779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27040" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{D191EDB1-F553-D84A-B803-B27A1F8FBA75}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{D191EDB1-F553-D84A-B803-B27A1F8FBA75}"/>
   </bookViews>
   <sheets>
     <sheet name="overall" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="25" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -812,12 +812,6 @@
     <t>14*3</t>
   </si>
   <si>
-    <t>3 to 2 and combined with the others</t>
-  </si>
-  <si>
-    <t>Count of 3 to 2 and combined with the others</t>
-  </si>
-  <si>
     <t>199-14=185</t>
   </si>
   <si>
@@ -825,6 +819,12 @@
   </si>
   <si>
     <t>more than 3</t>
+  </si>
+  <si>
+    <t>Thematic Relations</t>
+  </si>
+  <si>
+    <t>Counts</t>
   </si>
 </sst>
 </file>
@@ -880,7 +880,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -888,7 +888,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1649,10 +1648,10 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{63A041C4-9739-EE4D-9E2A-451E5AAB65D2}" name="PivotTable2" cacheId="25" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{63A041C4-9739-EE4D-9E2A-451E5AAB65D2}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A2:B34" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="1">
-    <pivotField name="3 to 2 and combined with the others" axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="descending">
+    <pivotField name="Thematic Relations" axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="descending">
       <items count="32">
         <item x="18"/>
         <item x="0"/>
@@ -1803,7 +1802,7 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of 3 to 2 and combined with the others" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Counts" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -2122,24 +2121,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="D1" s="6"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="6" t="s">
+      <c r="C1" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1" s="5"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -2797,10 +2796,10 @@
         <v>14</v>
       </c>
       <c r="H44" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
@@ -4993,17 +4992,17 @@
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3">
         <v>47</v>
       </c>
     </row>
@@ -5011,7 +5010,7 @@
       <c r="A4" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>19</v>
       </c>
     </row>
@@ -5019,7 +5018,7 @@
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>15</v>
       </c>
     </row>
@@ -5027,7 +5026,7 @@
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>13</v>
       </c>
     </row>
@@ -5035,7 +5034,7 @@
       <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>13</v>
       </c>
     </row>
@@ -5043,7 +5042,7 @@
       <c r="A8" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8">
         <v>9</v>
       </c>
     </row>
@@ -5051,7 +5050,7 @@
       <c r="A9" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9">
         <v>9</v>
       </c>
     </row>
@@ -5059,7 +5058,7 @@
       <c r="A10" t="s">
         <v>229</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10">
         <v>8</v>
       </c>
     </row>
@@ -5067,7 +5066,7 @@
       <c r="A11" t="s">
         <v>135</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11">
         <v>8</v>
       </c>
     </row>
@@ -5075,7 +5074,7 @@
       <c r="A12" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12">
         <v>7</v>
       </c>
     </row>
@@ -5083,7 +5082,7 @@
       <c r="A13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13">
         <v>7</v>
       </c>
     </row>
@@ -5091,7 +5090,7 @@
       <c r="A14" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14">
         <v>7</v>
       </c>
     </row>
@@ -5099,7 +5098,7 @@
       <c r="A15" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15">
         <v>7</v>
       </c>
     </row>
@@ -5107,7 +5106,7 @@
       <c r="A16" t="s">
         <v>103</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16">
         <v>6</v>
       </c>
     </row>
@@ -5115,7 +5114,7 @@
       <c r="A17" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17">
         <v>6</v>
       </c>
     </row>
@@ -5123,7 +5122,7 @@
       <c r="A18" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18">
         <v>5</v>
       </c>
     </row>
@@ -5131,7 +5130,7 @@
       <c r="A19" t="s">
         <v>147</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19">
         <v>5</v>
       </c>
     </row>
@@ -5139,7 +5138,7 @@
       <c r="A20" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20">
         <v>5</v>
       </c>
     </row>
@@ -5147,7 +5146,7 @@
       <c r="A21" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21">
         <v>5</v>
       </c>
     </row>
@@ -5155,7 +5154,7 @@
       <c r="A22" t="s">
         <v>120</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22">
         <v>4</v>
       </c>
     </row>
@@ -5163,7 +5162,7 @@
       <c r="A23" t="s">
         <v>89</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23">
         <v>3</v>
       </c>
     </row>
@@ -5171,7 +5170,7 @@
       <c r="A24" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24">
         <v>3</v>
       </c>
     </row>
@@ -5179,7 +5178,7 @@
       <c r="A25" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25">
         <v>3</v>
       </c>
     </row>
@@ -5187,7 +5186,7 @@
       <c r="A26" t="s">
         <v>65</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26">
         <v>3</v>
       </c>
     </row>
@@ -5195,7 +5194,7 @@
       <c r="A27" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27">
         <v>2</v>
       </c>
     </row>
@@ -5203,7 +5202,7 @@
       <c r="A28" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B28">
         <v>2</v>
       </c>
     </row>
@@ -5211,7 +5210,7 @@
       <c r="A29" t="s">
         <v>241</v>
       </c>
-      <c r="B29" s="5">
+      <c r="B29">
         <v>2</v>
       </c>
     </row>
@@ -5219,7 +5218,7 @@
       <c r="A30" t="s">
         <v>240</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30">
         <v>1</v>
       </c>
     </row>
@@ -5227,7 +5226,7 @@
       <c r="A31" t="s">
         <v>210</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31">
         <v>1</v>
       </c>
     </row>
@@ -5235,7 +5234,7 @@
       <c r="A32" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32">
         <v>1</v>
       </c>
     </row>
@@ -5243,7 +5242,7 @@
       <c r="A33" t="s">
         <v>116</v>
       </c>
-      <c r="B33" s="5">
+      <c r="B33">
         <v>1</v>
       </c>
     </row>
@@ -5251,7 +5250,7 @@
       <c r="A34" t="s">
         <v>253</v>
       </c>
-      <c r="B34" s="5">
+      <c r="B34">
         <v>227</v>
       </c>
     </row>

</xml_diff>